<commit_message>
feat: 支持禅道基于 RESTful API v2.0的实现
- 新增批量删除需求功能（支持 story/requirement/epic 三种类型）
- 重构服务层，拆分为独立的服务文件（story/requirement/epic）
- 修复 StoryListItem 结构体 JSON 解析问题（plan/estimate 字段类型）
- 新增 defaultReviewer 和 defaultModule 配置项
- 更新 README.md 和 EXCEL_FORMAT.md 文档并合并

兼容性说明：
- 最低支持版本：禅道 V21.7.9（开源版
- 低于此版本的 Token 获取机制存在差异，功能不可用
- 基于 RESTful API v2.0，需确保禅道已开启 API 功能
</commit_message>
<xml_diff>
--- a/requirements.xlsx
+++ b/requirements.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20916" windowHeight="6707"/>
+    <workbookView windowWidth="27870" windowHeight="14115"/>
   </bookViews>
   <sheets>
     <sheet name="requirements" sheetId="1" r:id="rId1"/>
@@ -1261,17 +1261,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:K5"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4" outlineLevelRow="4"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="13.5" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="17.5555555555556" customWidth="1"/>
-    <col min="2" max="2" width="11.8888888888889" customWidth="1"/>
-    <col min="3" max="4" width="10.7777777777778" customWidth="1"/>
-    <col min="5" max="5" width="34.7777777777778" customWidth="1"/>
-    <col min="6" max="6" width="16.2222222222222" customWidth="1"/>
-    <col min="7" max="7" width="18.5555555555556" customWidth="1"/>
-    <col min="8" max="8" width="23.1111111111111" customWidth="1"/>
+    <col min="1" max="1" width="17.5583333333333" customWidth="1"/>
+    <col min="2" max="2" width="11.8916666666667" customWidth="1"/>
+    <col min="3" max="4" width="10.775" customWidth="1"/>
+    <col min="5" max="5" width="34.775" customWidth="1"/>
+    <col min="6" max="6" width="16.225" customWidth="1"/>
+    <col min="7" max="7" width="18.5583333333333" customWidth="1"/>
+    <col min="8" max="8" width="23.1083333333333" customWidth="1"/>
     <col min="9" max="9" width="9.66666666666667" customWidth="1"/>
-    <col min="10" max="10" width="23.1111111111111" customWidth="1"/>
+    <col min="10" max="10" width="23.1083333333333" customWidth="1"/>
     <col min="11" max="11" width="41.3333333333333" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1315,7 +1315,7 @@
         <v>11</v>
       </c>
       <c r="B2">
-        <v>7</v>
+        <v>78</v>
       </c>
       <c r="C2">
         <v>2</v>
@@ -1344,7 +1344,7 @@
         <v>17</v>
       </c>
       <c r="B3">
-        <v>7</v>
+        <v>78</v>
       </c>
       <c r="C3">
         <v>3</v>
@@ -1379,7 +1379,7 @@
         <v>22</v>
       </c>
       <c r="B4">
-        <v>7</v>
+        <v>78</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -1402,7 +1402,7 @@
         <v>24</v>
       </c>
       <c r="B5">
-        <v>7</v>
+        <v>78</v>
       </c>
       <c r="C5">
         <v>1</v>

</xml_diff>